<commit_message>
Major change, adding optimisation routine
Includes an optimisation routine now to try and swap student's least favourite assignments with the most eligible other student.
</commit_message>
<xml_diff>
--- a/test_data/test_students_1.xlsx
+++ b/test_data/test_students_1.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E101"/>
+  <dimension ref="A1:E161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,34 +446,34 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Nina Becker</t>
+          <t>Sarah Bauer</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>Workshop10</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Workshop3</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
           <t>Workshop9</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Workshop2</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Workshop8</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Laura Weber</t>
+          <t>Leon Hofer</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -483,24 +483,24 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Workshop8</t>
+          <t>Workshop10</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Workshop2</t>
+          <t>Workshop9</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Workshop6</t>
+          <t>Workshop4</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Felix Koch</t>
+          <t>Felix Gruber</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -510,51 +510,51 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Workshop10</t>
+          <t>Workshop2</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Workshop9</t>
+          <t>Workshop3</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Workshop3</t>
+          <t>Workshop1</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Ben Schmidt</t>
+          <t>Lisa Richter</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Workshop4</t>
+          <t>Workshop1</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
+          <t>Workshop6</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
           <t>Workshop7</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Workshop10</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Felix Meyer</t>
+          <t>Sarah Friedl</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -564,24 +564,24 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Workshop1</t>
+          <t>Workshop9</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Workshop3</t>
+          <t>Workshop7</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Workshop9</t>
+          <t>Workshop8</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Emma Schmidt</t>
+          <t>Max Wolf</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -591,34 +591,34 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Workshop7</t>
+          <t>Workshop1</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Workshop1</t>
+          <t>Workshop3</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Workshop2</t>
+          <t>Workshop8</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Olivia Zimmermann</t>
+          <t>Hannah Weber</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Workshop9</t>
+          <t>Workshop2</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -628,68 +628,68 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Workshop10</t>
+          <t>Workshop4</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Emma Hartmann</t>
+          <t>Lisa Pichler</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Workshop2</t>
+          <t>Workshop8</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Workshop6</t>
+          <t>Workshop3</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Workshop8</t>
+          <t>Workshop7</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Ben Hartmann</t>
+          <t>Lisa Huber</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Workshop5</t>
+          <t>Workshop8</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Workshop10</t>
+          <t>Workshop1</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Workshop1</t>
+          <t>Workshop4</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Sara Klein</t>
+          <t>Matteo Weber</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -699,34 +699,34 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Workshop3</t>
+          <t>Workshop1</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Workshop1</t>
+          <t>Workshop6</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Workshop7</t>
+          <t>Workshop8</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Olivia Wolf</t>
+          <t>Laura Richter</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Workshop6</t>
+          <t>Workshop4</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -736,41 +736,41 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Workshop7</t>
+          <t>Workshop5</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Hannah Schneider</t>
+          <t>Sophie Wagner</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Workshop3</t>
+          <t>Workshop7</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
+          <t>Workshop1</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
           <t>Workshop5</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Workshop7</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Felix Wagner</t>
+          <t>Mia Gruber</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -780,159 +780,159 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Workshop6</t>
+          <t>Workshop8</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Workshop1</t>
+          <t>Workshop3</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Workshop10</t>
+          <t>Workshop2</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Max Weber</t>
+          <t>Ben Wagner</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Workshop8</t>
+          <t>Workshop1</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
+          <t>Workshop2</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
           <t>Workshop4</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Workshop7</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Noah Koch</t>
+          <t>Hannah Graf</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Workshop4</t>
+          <t>Workshop1</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Workshop6</t>
+          <t>Workshop3</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Workshop3</t>
+          <t>Workshop9</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Tim Müller</t>
+          <t>Sophie Fischer</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
+          <t>Workshop4</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
           <t>Workshop10</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Workshop6</t>
-        </is>
-      </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Workshop8</t>
+          <t>Workshop2</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Greta Schneider</t>
+          <t>Hannah Graf</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Workshop6</t>
+          <t>Workshop9</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Workshop8</t>
+          <t>Workshop2</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Workshop9</t>
+          <t>Workshop7</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Anna Becker</t>
+          <t>Mia Müller</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Workshop9</t>
+          <t>Workshop1</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Workshop8</t>
+          <t>Workshop4</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Workshop7</t>
+          <t>Workshop6</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Tim Schwarz</t>
+          <t>Katharina Müller</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -947,24 +947,24 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Workshop10</t>
+          <t>Workshop8</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Workshop3</t>
+          <t>Workshop5</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Jonas Wagner</t>
+          <t>David Kraus</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -974,46 +974,46 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Workshop4</t>
+          <t>Workshop5</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Workshop6</t>
+          <t>Workshop1</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Jonas Fischer</t>
+          <t>Paul Müller</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
+          <t>Workshop9</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Workshop4</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
           <t>Workshop7</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Workshop8</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>Workshop10</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Tim Hartmann</t>
+          <t>Nina Friedl</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1023,24 +1023,24 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Workshop2</t>
+          <t>Workshop10</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Workshop6</t>
+          <t>Workshop3</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Workshop8</t>
+          <t>Workshop6</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Noah Krüger</t>
+          <t>Lena Kraus</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1050,105 +1050,105 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Workshop6</t>
+          <t>Workshop3</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Workshop1</t>
+          <t>Workshop4</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Workshop8</t>
+          <t>Workshop9</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Mia Schwarz</t>
+          <t>Mia Steiner</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Workshop2</t>
+          <t>Workshop5</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Workshop3</t>
+          <t>Workshop10</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Workshop4</t>
+          <t>Workshop1</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Sara Wolf</t>
+          <t>Katharina Wolf</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Workshop10</t>
+          <t>Workshop5</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Workshop8</t>
+          <t>Workshop4</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Workshop7</t>
+          <t>Workshop1</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Hannah Neumann</t>
+          <t>Paul Meyer</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Workshop7</t>
+          <t>Workshop4</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Workshop10</t>
+          <t>Workshop8</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Workshop1</t>
+          <t>Workshop3</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Paul Müller</t>
+          <t>Jakob Berger</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1163,46 +1163,46 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Workshop6</t>
+          <t>Workshop8</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Workshop5</t>
+          <t>Workshop6</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Nina Krüger</t>
+          <t>Elias Berger</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Workshop2</t>
+          <t>Workshop4</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Workshop3</t>
+          <t>Workshop1</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Workshop8</t>
+          <t>Workshop6</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Laura Müller</t>
+          <t>Marie Lang</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1212,24 +1212,24 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Workshop3</t>
+          <t>Workshop10</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
+          <t>Workshop5</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
           <t>Workshop9</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>Workshop1</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Leon Lange</t>
+          <t>Moritz Leitner</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1249,14 +1249,14 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Workshop6</t>
+          <t>Workshop10</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Mia Schneider</t>
+          <t>Anna Kraus</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1266,17 +1266,17 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Workshop5</t>
+          <t>Workshop8</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Workshop6</t>
+          <t>Workshop1</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Workshop4</t>
+          <t>Workshop6</t>
         </is>
       </c>
     </row>
@@ -1293,24 +1293,24 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Workshop8</t>
+          <t>Workshop7</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Workshop6</t>
+          <t>Workshop2</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Workshop7</t>
+          <t>Workshop5</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Laura Hoffmann</t>
+          <t>Jonas Hofer</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1320,24 +1320,24 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Workshop9</t>
+          <t>Workshop8</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Workshop7</t>
+          <t>Workshop2</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Workshop6</t>
+          <t>Workshop10</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Nina Zimmermann</t>
+          <t>Elias Lang</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1347,7 +1347,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Workshop4</t>
+          <t>Workshop9</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1357,46 +1357,46 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Workshop3</t>
+          <t>Workshop5</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Felix Hartmann</t>
+          <t>Tim Fischer</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
+          <t>Workshop1</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
           <t>Workshop5</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>Workshop2</t>
-        </is>
-      </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Workshop6</t>
+          <t>Workshop10</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Felix Hoffmann</t>
+          <t>Felix Fischer</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1406,46 +1406,46 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Workshop2</t>
+          <t>Workshop1</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Workshop4</t>
+          <t>Workshop8</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Max Lange</t>
+          <t>Lisa Berger</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Workshop3</t>
+          <t>Workshop7</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Workshop7</t>
+          <t>Workshop8</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Workshop9</t>
+          <t>Workshop10</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Lena Fischer</t>
+          <t>Clara Wolf</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1455,51 +1455,51 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
+          <t>Workshop9</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Workshop10</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
           <t>Workshop4</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>Workshop3</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>Workshop1</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Paul Krüger</t>
+          <t>Fabian Graf</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Workshop3</t>
+          <t>Workshop9</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Workshop4</t>
+          <t>Workshop7</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Workshop9</t>
+          <t>Workshop1</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Hannah Fischer</t>
+          <t>Max Huber</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1514,7 +1514,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Workshop2</t>
+          <t>Workshop10</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -1526,61 +1526,61 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Mia Schwarz</t>
+          <t>Mia Schmidt</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Workshop6</t>
+          <t>Workshop5</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Workshop5</t>
+          <t>Workshop3</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Workshop10</t>
+          <t>Workshop6</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Emma Lange</t>
+          <t>Sophie Richter</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Workshop4</t>
+          <t>Workshop6</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Workshop7</t>
+          <t>Workshop8</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Workshop8</t>
+          <t>Workshop1</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Laura Krüger</t>
+          <t>Hannah Maier</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1590,24 +1590,24 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Workshop7</t>
+          <t>Workshop3</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Workshop10</t>
+          <t>Workshop1</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Workshop2</t>
+          <t>Workshop9</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Emma Hartmann</t>
+          <t>Felix Weber</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1617,51 +1617,51 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Workshop6</t>
+          <t>Workshop5</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Workshop9</t>
+          <t>Workshop7</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Workshop8</t>
+          <t>Workshop2</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Anna Schneider</t>
+          <t>Leon Maier</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Workshop4</t>
+          <t>Workshop7</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Workshop5</t>
+          <t>Workshop2</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Workshop2</t>
+          <t>Workshop9</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Paul Hartmann</t>
+          <t>Simon Auer</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1671,12 +1671,12 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Workshop6</t>
+          <t>Workshop2</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Workshop10</t>
+          <t>Workshop3</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -1688,12 +1688,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Lena Weber</t>
+          <t>Felix Meyer</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -1703,73 +1703,73 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
+          <t>Workshop3</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
           <t>Workshop10</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>Workshop4</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Max Schwarz</t>
+          <t>Fabian Graf</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
+          <t>Workshop1</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
           <t>Workshop7</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>Workshop10</t>
-        </is>
-      </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Workshop1</t>
+          <t>Workshop9</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Tim Lange</t>
+          <t>Felix Weber</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Workshop3</t>
+          <t>Workshop9</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Workshop6</t>
+          <t>Workshop4</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Workshop10</t>
+          <t>Workshop5</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Hannah Schulz</t>
+          <t>Moritz Wagner</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1779,56 +1779,56 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
+          <t>Workshop2</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
           <t>Workshop5</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>Workshop10</t>
-        </is>
-      </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Workshop1</t>
+          <t>Workshop8</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Nina Fischer</t>
+          <t>Simon Hofer</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Workshop8</t>
+          <t>Workshop1</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Workshop9</t>
+          <t>Workshop6</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Workshop6</t>
+          <t>Workshop2</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Olivia Klein</t>
+          <t>Sarah Hofer</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -1838,181 +1838,181 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Workshop4</t>
+          <t>Workshop2</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Workshop5</t>
+          <t>Workshop3</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Clara Lange</t>
+          <t>Leon Auer</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Workshop2</t>
+          <t>Workshop6</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Workshop5</t>
+          <t>Workshop8</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Workshop8</t>
+          <t>Workshop3</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Sara Schmidt</t>
+          <t>Lisa Maier</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Workshop2</t>
+          <t>Workshop9</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Workshop8</t>
+          <t>Workshop6</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Workshop6</t>
+          <t>Workshop5</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Paul Neumann</t>
+          <t>Julia Pichler</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Workshop1</t>
+          <t>Workshop5</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Workshop10</t>
+          <t>Workshop4</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Workshop3</t>
+          <t>Workshop8</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Jonas Schneider</t>
+          <t>Simon Richter</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Workshop10</t>
+          <t>Workshop6</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Workshop6</t>
+          <t>Workshop9</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Workshop3</t>
+          <t>Workshop4</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Mia Hoffmann</t>
+          <t>Laura Schmidt</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Workshop6</t>
+          <t>Workshop2</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
+          <t>Workshop8</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
           <t>Workshop10</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>Workshop1</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Hannah Wagner</t>
+          <t>Tim Leitner</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Workshop7</t>
+          <t>Workshop9</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Workshop2</t>
+          <t>Workshop5</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Workshop9</t>
+          <t>Workshop4</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Lena Schmidt</t>
+          <t>Marie Wolf</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2022,24 +2022,24 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Workshop7</t>
+          <t>Workshop3</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Workshop6</t>
+          <t>Workshop5</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Workshop8</t>
+          <t>Workshop6</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Max Schulz</t>
+          <t>Simon Weber</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2049,24 +2049,24 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Workshop6</t>
+          <t>Workshop4</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Workshop2</t>
+          <t>Workshop6</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Workshop10</t>
+          <t>Workshop8</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Emma Klein</t>
+          <t>Anna Steiner</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2076,24 +2076,24 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Workshop10</t>
+          <t>Workshop9</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Workshop8</t>
+          <t>Workshop6</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Workshop1</t>
+          <t>Workshop2</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Clara Koch</t>
+          <t>Emma Gruber</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2103,51 +2103,51 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Workshop2</t>
+          <t>Workshop1</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Workshop10</t>
+          <t>Workshop3</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Workshop4</t>
+          <t>Workshop5</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Nina Krüger</t>
+          <t>Fabian Wolf</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Workshop3</t>
+          <t>Workshop6</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Workshop9</t>
+          <t>Workshop8</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Workshop5</t>
+          <t>Workshop4</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>David Becker</t>
+          <t>David Schmidt</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2157,24 +2157,24 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Workshop7</t>
+          <t>Workshop3</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
+          <t>Workshop6</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
           <t>Workshop5</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>Workshop2</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Greta Wagner</t>
+          <t>Tim Huber</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -2184,24 +2184,24 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Workshop10</t>
+          <t>Workshop3</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Workshop1</t>
+          <t>Workshop2</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Workshop4</t>
+          <t>Workshop1</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Olivia Müller</t>
+          <t>Sarah Wolf</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2211,51 +2211,51 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
+          <t>Workshop6</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
           <t>Workshop8</t>
         </is>
       </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>Workshop1</t>
-        </is>
-      </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Workshop3</t>
+          <t>Workshop1</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Leon Hartmann</t>
+          <t>Emma Gruber</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Workshop10</t>
+          <t>Workshop9</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Workshop3</t>
+          <t>Workshop4</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Workshop2</t>
+          <t>Workshop3</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Tim Krüger</t>
+          <t>David Weber</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2265,51 +2265,51 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Workshop5</t>
+          <t>Workshop6</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Workshop1</t>
+          <t>Workshop2</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Workshop3</t>
+          <t>Workshop1</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Laura Zimmermann</t>
+          <t>Nina Leitner</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Workshop1</t>
+          <t>Workshop7</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Workshop3</t>
+          <t>Workshop8</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Workshop2</t>
+          <t>Workshop5</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Jonas Schulz</t>
+          <t>Elias Graf</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -2319,83 +2319,83 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
+          <t>Workshop6</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Workshop10</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
           <t>Workshop5</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>Workshop8</t>
-        </is>
-      </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>Workshop6</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Tim Hartmann</t>
+          <t>Lukas Maier</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Workshop3</t>
+          <t>Workshop9</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Workshop9</t>
+          <t>Workshop3</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Workshop8</t>
+          <t>Workshop4</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Tim Meyer</t>
+          <t>Amelie Koch</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Workshop4</t>
+          <t>Workshop2</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Workshop2</t>
+          <t>Workshop6</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Workshop3</t>
+          <t>Workshop8</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Jonas Klein</t>
+          <t>Jonas Bauer</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -2405,100 +2405,100 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Workshop8</t>
+          <t>Workshop7</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Workshop9</t>
+          <t>Workshop3</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Ben Schulz</t>
+          <t>Emma Meyer</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Workshop3</t>
+          <t>Workshop2</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
+          <t>Workshop3</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
           <t>Workshop10</t>
-        </is>
-      </c>
-      <c r="E75" t="inlineStr">
-        <is>
-          <t>Workshop1</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Mia Klein</t>
+          <t>Nina Graf</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Workshop4</t>
+          <t>Workshop5</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Workshop3</t>
+          <t>Workshop2</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Workshop9</t>
+          <t>Workshop7</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Sara Neumann</t>
+          <t>Clara Berger</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Workshop7</t>
+          <t>Workshop5</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Workshop4</t>
+          <t>Workshop2</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Workshop5</t>
+          <t>Workshop8</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Max Müller</t>
+          <t>Elias Hofer</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2508,132 +2508,132 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Workshop5</t>
+          <t>Workshop7</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Workshop6</t>
+          <t>Workshop9</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Workshop8</t>
+          <t>Workshop3</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Felix Neumann</t>
+          <t>Katharina Wolf</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Workshop1</t>
+          <t>Workshop3</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Workshop3</t>
+          <t>Workshop6</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Workshop10</t>
+          <t>Workshop1</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Nina Wolf</t>
+          <t>Mia Fischer</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Workshop7</t>
+          <t>Workshop8</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Workshop2</t>
+          <t>Workshop6</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Workshop10</t>
+          <t>Workshop9</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Greta Müller</t>
+          <t>Mia Wagner</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Workshop4</t>
+          <t>Workshop3</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Workshop6</t>
+          <t>Workshop2</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Workshop2</t>
+          <t>Workshop8</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Nina Neumann</t>
+          <t>Hannah Weber</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Workshop6</t>
+          <t>Workshop9</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Workshop1</t>
+          <t>Workshop5</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Workshop9</t>
+          <t>Workshop6</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Greta Hartmann</t>
+          <t>Julia Richter</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2643,24 +2643,24 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Workshop4</t>
+          <t>Workshop3</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Workshop2</t>
+          <t>Workshop9</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Workshop10</t>
+          <t>Workshop2</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Emma Zimmermann</t>
+          <t>Hannah Wolf</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2670,24 +2670,24 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Workshop1</t>
+          <t>Workshop2</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Workshop10</t>
+          <t>Workshop1</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Workshop5</t>
+          <t>Workshop4</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Laura Zimmermann</t>
+          <t>Emma Müller</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -2697,51 +2697,51 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Workshop9</t>
+          <t>Workshop3</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Workshop10</t>
+          <t>Workshop7</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Workshop8</t>
+          <t>Workshop2</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Mia Weber</t>
+          <t>Lukas Kraus</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Workshop9</t>
+          <t>Workshop10</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Workshop5</t>
+          <t>Workshop8</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Workshop3</t>
+          <t>Workshop4</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Paul Weber</t>
+          <t>Lukas Wagner</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2751,24 +2751,24 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
+          <t>Workshop6</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Workshop2</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
           <t>Workshop7</t>
-        </is>
-      </c>
-      <c r="D87" t="inlineStr">
-        <is>
-          <t>Workshop6</t>
-        </is>
-      </c>
-      <c r="E87" t="inlineStr">
-        <is>
-          <t>Workshop4</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Anna Lange</t>
+          <t>Ben Schmidt</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2778,105 +2778,105 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Workshop6</t>
+          <t>Workshop3</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Workshop8</t>
+          <t>Workshop1</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Workshop4</t>
+          <t>Workshop5</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Emma Zimmermann</t>
+          <t>Lisa Schmidt</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Workshop4</t>
+          <t>Workshop8</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Workshop7</t>
+          <t>Workshop9</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Workshop6</t>
+          <t>Workshop2</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Mia Hoffmann</t>
+          <t>Leon Berger</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
+          <t>Workshop3</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Workshop8</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
           <t>Workshop10</t>
-        </is>
-      </c>
-      <c r="D90" t="inlineStr">
-        <is>
-          <t>Workshop3</t>
-        </is>
-      </c>
-      <c r="E90" t="inlineStr">
-        <is>
-          <t>Workshop9</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Nina Zimmermann</t>
+          <t>Max Wagner</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Workshop6</t>
+          <t>Workshop1</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Workshop5</t>
+          <t>Workshop2</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Workshop9</t>
+          <t>Workshop10</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Mia Hartmann</t>
+          <t>Tim Wolf</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2886,39 +2886,39 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Workshop2</t>
+          <t>Workshop3</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Workshop10</t>
+          <t>Workshop6</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Workshop8</t>
+          <t>Workshop1</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Tim Wolf</t>
+          <t>David Maier</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Workshop2</t>
+          <t>Workshop3</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Workshop9</t>
+          <t>Workshop2</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -2930,7 +2930,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Leon Lange</t>
+          <t>Clara Koch</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2940,24 +2940,24 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Workshop3</t>
+          <t>Workshop1</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Workshop2</t>
+          <t>Workshop8</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Workshop7</t>
+          <t>Workshop4</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Noah Müller</t>
+          <t>Jonas Huber</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2967,24 +2967,24 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
+          <t>Workshop6</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
           <t>Workshop9</t>
         </is>
       </c>
-      <c r="D95" t="inlineStr">
-        <is>
-          <t>Workshop2</t>
-        </is>
-      </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Workshop6</t>
+          <t>Workshop8</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Ben Schwarz</t>
+          <t>Amelie Gruber</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2994,24 +2994,24 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Workshop8</t>
+          <t>Workshop4</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Workshop10</t>
+          <t>Workshop3</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Workshop9</t>
+          <t>Workshop5</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Clara Weber</t>
+          <t>Felix Huber</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -3026,19 +3026,19 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Workshop6</t>
+          <t>Workshop2</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Workshop8</t>
+          <t>Workshop1</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Mia Schulz</t>
+          <t>Leon Graf</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -3048,7 +3048,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Workshop6</t>
+          <t>Workshop5</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -3058,41 +3058,41 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Workshop2</t>
+          <t>Workshop10</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Tim Weber</t>
+          <t>Jonas Wagner</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Workshop10</t>
+          <t>Workshop5</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Workshop4</t>
+          <t>Workshop6</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Workshop3</t>
+          <t>Workshop8</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Lena Hartmann</t>
+          <t>David Schmidt</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -3102,24 +3102,24 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Workshop6</t>
+          <t>Workshop10</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Workshop10</t>
+          <t>Workshop6</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Workshop5</t>
+          <t>Workshop1</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Leon Hartmann</t>
+          <t>Jonas Auer</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -3129,17 +3129,1637 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
+          <t>Workshop10</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Workshop4</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Workshop3</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Anna Meyer</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Workshop2</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Workshop10</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Workshop3</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Emma Bauer</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Workshop9</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Workshop3</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Workshop2</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Marie Friedl</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Workshop4</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Workshop1</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Workshop10</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Mia Wolf</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Workshop2</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Workshop6</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Workshop4</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Anna Leitner</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Workshop3</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Workshop1</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Workshop7</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Sophie Bauer</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
           <t>Workshop8</t>
         </is>
       </c>
-      <c r="D101" t="inlineStr">
-        <is>
-          <t>Workshop1</t>
-        </is>
-      </c>
-      <c r="E101" t="inlineStr">
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Workshop1</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Workshop4</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Moritz Hofer</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
         <is>
           <t>Workshop5</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Workshop1</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Workshop4</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Tim Schwarz</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Workshop10</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Workshop5</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Workshop4</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Amelie Fischer</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Workshop7</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Workshop4</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Workshop9</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Clara Gruber</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Workshop2</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Workshop9</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Workshop3</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Lisa Schmidt</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Workshop4</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Workshop7</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Workshop5</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Lisa Müller</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Workshop9</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Workshop1</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Workshop3</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Marie Lang</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Workshop5</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Workshop3</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Workshop2</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Noah Fischer</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Workshop6</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Workshop7</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>Workshop3</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Tim Leitner</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Workshop7</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Workshop8</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Workshop3</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Laura Wagner</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Workshop3</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Workshop2</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>Workshop5</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Katharina Hofer</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Workshop7</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Workshop10</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>Workshop5</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Amelie Gruber</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Workshop2</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Workshop6</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>Workshop8</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Anna Bauer</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Workshop5</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Workshop8</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Workshop1</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Felix Meyer</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Workshop5</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Workshop1</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Workshop9</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Lea Leitner</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Workshop4</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Workshop6</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>Workshop3</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Lukas Bauer</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Workshop9</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Workshop3</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>Workshop6</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Marie Schwarz</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Workshop10</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Workshop4</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>Workshop3</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Nina Schmidt</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Workshop2</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Workshop6</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>Workshop1</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Lukas Hofer</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Workshop8</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Workshop1</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>Workshop7</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>David Graf</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Workshop4</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Workshop3</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Workshop9</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Max Koch</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Workshop7</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Workshop4</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>Workshop5</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Lena Maier</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Workshop9</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Workshop10</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>Workshop5</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Lisa Meyer</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Workshop7</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Workshop2</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>Workshop5</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Lena Kraus</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Workshop6</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Workshop9</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>Workshop8</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Elias Lang</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Workshop7</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Workshop10</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>Workshop1</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Nina Maier</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Workshop5</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Workshop1</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>Workshop9</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Fabian Weber</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Workshop9</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Workshop8</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>Workshop3</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Fabian Bauer</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Workshop9</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Workshop4</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>Workshop3</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Ben Wagner</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Workshop5</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Workshop8</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>Workshop10</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Mia Bauer</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Workshop2</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Workshop10</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>Workshop5</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Laura Gruber</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Workshop1</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Workshop6</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>Workshop8</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Matteo Schmidt</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Workshop5</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Workshop3</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>Workshop1</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>Lisa Koch</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Workshop7</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>Workshop2</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>Workshop1</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>Paul Kraus</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Workshop2</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Workshop7</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>Workshop3</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Hannah Wolf</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Workshop6</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Workshop7</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>Workshop2</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>Nina Wagner</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Workshop6</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Workshop2</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>Workshop3</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>Sarah Schmidt</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Workshop6</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Workshop10</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>Workshop1</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Tim Kraus</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Workshop8</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Workshop10</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>Workshop9</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Elias Graf</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Workshop4</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Workshop6</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>Workshop9</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>Clara Friedl</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Workshop4</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Workshop7</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>Workshop8</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>Moritz Gruber</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Workshop3</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Workshop7</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>Workshop2</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>Mia Friedl</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Workshop6</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Workshop3</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>Workshop9</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>Emma Steiner</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Workshop3</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Workshop10</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>Workshop6</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Moritz Fischer</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Workshop5</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Workshop6</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>Workshop4</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>Elias Friedl</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Workshop7</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Workshop9</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>Workshop8</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>Laura Koch</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Workshop1</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Workshop2</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>Workshop10</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>Hannah Gruber</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Workshop6</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Workshop5</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>Workshop7</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>Amelie Müller</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Workshop7</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Workshop8</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>Workshop6</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>Laura Berger</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Workshop6</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Workshop4</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>Workshop3</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>Emma Koch</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Workshop10</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Workshop1</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>Workshop2</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>Fabian Berger</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Workshop1</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Workshop4</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>Workshop6</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>Max Graf</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Workshop6</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Workshop5</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>Workshop2</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>Marie Weber</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Workshop2</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Workshop5</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>Workshop9</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>Simon Berger</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Workshop1</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>Workshop9</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>Workshop4</t>
         </is>
       </c>
     </row>

</xml_diff>